<commit_message>
[Update] : validation duplicat id_rup
</commit_message>
<xml_diff>
--- a/public/uploads/template/Template_Form_Daftar_Pemenang.xlsx
+++ b/public/uploads/template/Template_Form_Daftar_Pemenang.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HELMY\PROJECT\Pengadaan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HELMY\PROJECT\project-root-rbac\public\uploads\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6FC6BD7-2714-4E55-8E0A-580B44E4D4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48604D65-AAE0-4680-9739-7A23CEDACB8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CB47FC0-B818-464B-9049-99572A7EB9D8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t>No</t>
   </si>
@@ -128,6 +128,24 @@
   </si>
   <si>
     <t>PW 11-2025, Pengawasan Teknis Preservasi Jalan Provinsi Jawa Barat -1</t>
+  </si>
+  <si>
+    <t>ID RUP</t>
+  </si>
+  <si>
+    <t>0000000001</t>
+  </si>
+  <si>
+    <t>0000000003</t>
+  </si>
+  <si>
+    <t>0000000005</t>
+  </si>
+  <si>
+    <t>0000000002</t>
+  </si>
+  <si>
+    <t>0000000004</t>
   </si>
 </sst>
 </file>
@@ -138,7 +156,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="[$Rp-3809]#,##0.00;\-[$Rp-3809]#,##0.00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -155,6 +173,11 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -180,7 +203,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -222,6 +245,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -438,310 +468,330 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD805072-6504-46FC-A5EB-1059C7837CED}">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.44140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" customWidth="1"/>
-    <col min="7" max="7" width="20.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="9.6640625" customWidth="1"/>
-    <col min="10" max="10" width="15" style="14" customWidth="1"/>
-    <col min="11" max="11" width="13.109375" style="14" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7" customWidth="1"/>
-    <col min="13" max="13" width="19.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.77734375" style="14" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="74.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="34" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.77734375" style="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="9.6640625" customWidth="1"/>
+    <col min="11" max="11" width="15" style="14" customWidth="1"/>
+    <col min="12" max="12" width="13.109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7" customWidth="1"/>
+    <col min="14" max="14" width="19.6640625" style="14" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.77734375" style="14" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="74.44140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="6" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="6" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="P1" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="92.4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="92.4" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="8">
+      <c r="D2" s="8">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="1">
-        <v>2</v>
-      </c>
-      <c r="F2" s="4">
+      <c r="F2" s="1">
+        <v>2</v>
+      </c>
+      <c r="G2" s="4">
         <v>0.87570000000000003</v>
       </c>
-      <c r="G2" s="9">
+      <c r="H2" s="9">
         <v>1189998412</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="1">
+      <c r="J2" s="1">
         <v>21</v>
       </c>
-      <c r="J2" s="12">
+      <c r="K2" s="12">
         <v>45840</v>
       </c>
-      <c r="K2" s="12">
+      <c r="L2" s="12">
         <v>45861</v>
       </c>
-      <c r="L2" s="1">
-        <v>2</v>
-      </c>
-      <c r="M2" s="12">
+      <c r="M2" s="1">
+        <v>2</v>
+      </c>
+      <c r="N2" s="12">
         <v>45863</v>
       </c>
-      <c r="N2" s="12">
+      <c r="O2" s="12">
         <v>45861</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="1">
-        <v>2</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="1">
+        <v>2</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="1">
-        <v>2</v>
-      </c>
-      <c r="F3" s="4">
+      <c r="F3" s="1">
+        <v>2</v>
+      </c>
+      <c r="G3" s="4">
         <v>0.82489999999999997</v>
       </c>
-      <c r="G3" s="10">
+      <c r="H3" s="10">
         <v>5211169503</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="1">
+      <c r="J3" s="1">
         <v>47</v>
       </c>
-      <c r="J3" s="12">
+      <c r="K3" s="12">
         <v>45842</v>
       </c>
-      <c r="K3" s="12">
+      <c r="L3" s="12">
         <v>45889</v>
       </c>
-      <c r="L3" s="1">
+      <c r="M3" s="1">
         <v>1</v>
       </c>
-      <c r="M3" s="12">
+      <c r="N3" s="12">
         <v>45884</v>
       </c>
-      <c r="N3" s="12">
+      <c r="O3" s="12">
         <v>45889</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="P3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="1">
-        <v>2</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="1">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="1">
-        <v>2</v>
-      </c>
-      <c r="F4" s="4">
+      <c r="F4" s="1">
+        <v>2</v>
+      </c>
+      <c r="G4" s="4">
         <v>0.82569999999999999</v>
       </c>
-      <c r="G4" s="10">
+      <c r="H4" s="10">
         <v>4079248779</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="1">
+      <c r="J4" s="1">
         <v>47</v>
       </c>
-      <c r="J4" s="12">
+      <c r="K4" s="12">
         <v>45842</v>
       </c>
-      <c r="K4" s="12">
+      <c r="L4" s="12">
         <v>45889</v>
       </c>
-      <c r="L4" s="1">
+      <c r="M4" s="1">
         <v>1</v>
       </c>
-      <c r="M4" s="12">
+      <c r="N4" s="12">
         <v>45884</v>
       </c>
-      <c r="N4" s="12">
+      <c r="O4" s="12">
         <v>45889</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="P4" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="1">
-        <v>2</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="1">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="1">
-        <v>2</v>
-      </c>
-      <c r="F5" s="4">
+      <c r="F5" s="1">
+        <v>2</v>
+      </c>
+      <c r="G5" s="4">
         <v>0.8</v>
       </c>
-      <c r="G5" s="10">
+      <c r="H5" s="10">
         <v>179943326572.32001</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="1">
+      <c r="J5" s="1">
         <v>76</v>
       </c>
-      <c r="J5" s="12">
+      <c r="K5" s="12">
         <v>45849</v>
       </c>
-      <c r="K5" s="12">
+      <c r="L5" s="12">
         <v>45925</v>
       </c>
-      <c r="L5" s="1">
-        <v>2</v>
-      </c>
-      <c r="M5" s="12">
+      <c r="M5" s="1">
+        <v>2</v>
+      </c>
+      <c r="N5" s="12">
         <v>45883</v>
       </c>
-      <c r="N5" s="12">
+      <c r="O5" s="12">
         <v>45889</v>
       </c>
-      <c r="O5" s="3" t="s">
+      <c r="P5" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="1">
-        <v>2</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="1">
+        <v>2</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="1">
+      <c r="F6" s="1">
         <v>1</v>
       </c>
-      <c r="F6" s="4">
+      <c r="G6" s="4">
         <v>0.9587</v>
       </c>
-      <c r="G6" s="10">
+      <c r="H6" s="10">
         <v>2441804640</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="1">
+      <c r="J6" s="1">
         <v>13</v>
       </c>
-      <c r="J6" s="12">
+      <c r="K6" s="12">
         <v>45853</v>
       </c>
-      <c r="K6" s="12">
+      <c r="L6" s="12">
         <v>45866</v>
       </c>
-      <c r="L6" s="1">
+      <c r="M6" s="1">
         <v>1</v>
-      </c>
-      <c r="M6" s="12">
-        <v>45889</v>
       </c>
       <c r="N6" s="12">
         <v>45889</v>
       </c>
-      <c r="O6" s="3"/>
+      <c r="O6" s="12">
+        <v>45889</v>
+      </c>
+      <c r="P6" s="3"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="J7" s="13"/>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="K7" s="13"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>